<commit_message>
change project planning structure
</commit_message>
<xml_diff>
--- a/Documentation/project-plan.xlsx
+++ b/Documentation/project-plan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ebiru\code\Informatik-2.Jahr\IPT6.1\IPT6.1-Productivity-Game\Documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanji\Documents\GitHub\IPT7.1-Projekt-Kick-Off\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26A8F9F7-72A1-4B69-968E-D610224F13F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4CCFDD6-667C-4AE1-9915-93A497954C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Idea Planner" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,8 @@
   <definedNames>
     <definedName name="ColumnTitle1">Tasks[[#Headers],[ Task Status Indicator]]</definedName>
     <definedName name="ColumnTitleRegion1..G5.1">'Idea Planner'!$B$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Idea Planner'!$6:$6</definedName>
     <definedName name="PlanDueDate">'Idea Planner'!$E$3</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Idea Planner'!$6:$6</definedName>
     <definedName name="RowTitleRegion1..E3">'Idea Planner'!$D$2</definedName>
     <definedName name="RowTitleRegion2..G3">'Idea Planner'!$F$2</definedName>
   </definedNames>
@@ -840,26 +840,26 @@
     </xf>
   </cellXfs>
   <cellStyles count="20">
-    <cellStyle name="Calculation" xfId="16" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Berechnung" xfId="16" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Besuchter Hyperlink" xfId="6" builtinId="9" customBuiltin="1"/>
     <cellStyle name="Center aligned" xfId="9" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="Comma" xfId="10" builtinId="3" customBuiltin="1"/>
-    <cellStyle name="Comma [0]" xfId="11" builtinId="6" customBuiltin="1"/>
-    <cellStyle name="Currency" xfId="12" builtinId="4" customBuiltin="1"/>
-    <cellStyle name="Currency [0]" xfId="13" builtinId="7" customBuiltin="1"/>
+    <cellStyle name="Dezimal [0]" xfId="11" builtinId="6" customBuiltin="1"/>
     <cellStyle name="Due Date" xfId="18" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Explanatory Text" xfId="7" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Hyperlink" xfId="5" builtinId="8" customBuiltin="1"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
-    <cellStyle name="Per cent" xfId="14" builtinId="5" customBuiltin="1"/>
+    <cellStyle name="Erklärender Text" xfId="7" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Komma" xfId="10" builtinId="3" customBuiltin="1"/>
+    <cellStyle name="Link" xfId="5" builtinId="8" customBuiltin="1"/>
     <cellStyle name="Plan Due Date" xfId="8" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="Prozent" xfId="14" builtinId="5" customBuiltin="1"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0" customBuiltin="1"/>
     <cellStyle name="Status Icon Text" xfId="19" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
     <cellStyle name="Task Indicator" xfId="17" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Überschrift" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Überschrift 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Überschrift 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Überschrift 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Überschrift 4" xfId="15" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Währung" xfId="12" builtinId="4" customBuiltin="1"/>
+    <cellStyle name="Währung [0]" xfId="13" builtinId="7" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="11">
     <dxf>
@@ -1336,23 +1336,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:G133"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.54296875" customWidth="1"/>
+    <col min="1" max="1" width="2.5546875" customWidth="1"/>
     <col min="2" max="2" width="1" customWidth="1"/>
-    <col min="3" max="3" width="42.54296875" customWidth="1"/>
-    <col min="4" max="4" width="18.54296875" customWidth="1"/>
-    <col min="5" max="5" width="22.54296875" customWidth="1"/>
+    <col min="3" max="3" width="42.5546875" customWidth="1"/>
+    <col min="4" max="4" width="18.5546875" customWidth="1"/>
+    <col min="5" max="5" width="22.5546875" customWidth="1"/>
     <col min="6" max="6" width="31" customWidth="1"/>
-    <col min="7" max="7" width="43.453125" customWidth="1"/>
-    <col min="8" max="8" width="2.54296875" customWidth="1"/>
+    <col min="7" max="7" width="43.44140625" customWidth="1"/>
+    <col min="8" max="8" width="2.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="33"/>
       <c r="C1" s="33"/>
     </row>
-    <row r="2" spans="2:7" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:7" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="34" t="s">
         <v>0</v>
       </c>
@@ -1366,7 +1366,7 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="2:7" ht="33" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:7" ht="33" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="34"/>
       <c r="C3" s="34"/>
       <c r="D3" s="10" t="s">
@@ -1382,7 +1382,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="2:7" ht="28.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:7" ht="28.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="B4" s="35" t="s">
         <v>3</v>
       </c>
@@ -1394,7 +1394,7 @@
       <c r="F4" s="35"/>
       <c r="G4" s="35"/>
     </row>
-    <row r="5" spans="2:7" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:7" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="36" t="s">
         <v>145</v>
       </c>
@@ -1406,7 +1406,7 @@
       <c r="F5" s="36"/>
       <c r="G5" s="36"/>
     </row>
-    <row r="6" spans="2:7" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:7" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
@@ -1426,7 +1426,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="8" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="G7" s="26"/>
     </row>
-    <row r="8" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="8">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1464,7 +1464,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="8">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1486,7 +1486,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="8">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1508,7 +1508,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1530,7 +1530,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="12" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="G12" s="28"/>
     </row>
-    <row r="13" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1568,7 +1568,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="14" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1590,7 +1590,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="15" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1612,7 +1612,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="16" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1634,7 +1634,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1656,7 +1656,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="G18" s="29"/>
     </row>
-    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1694,7 +1694,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1716,7 +1716,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1738,7 +1738,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1760,7 +1760,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>1</v>
@@ -1782,7 +1782,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>0</v>
@@ -1804,7 +1804,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>0</v>
@@ -1826,7 +1826,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="G26" s="25"/>
     </row>
-    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>0</v>
@@ -1864,7 +1864,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>0</v>
@@ -1886,7 +1886,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1902,7 +1902,7 @@
       </c>
       <c r="G29" s="25"/>
     </row>
-    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -1924,7 +1924,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -1940,7 +1940,7 @@
       </c>
       <c r="G31" s="17"/>
     </row>
-    <row r="32" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -1962,7 +1962,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -1984,7 +1984,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2006,7 +2006,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="35" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2028,7 +2028,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="36" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="G36" s="26"/>
     </row>
-    <row r="37" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2066,7 +2066,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="38" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2088,7 +2088,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="39" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2110,7 +2110,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="40" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="G40" s="26"/>
     </row>
-    <row r="41" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2148,7 +2148,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="42" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2170,7 +2170,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="43" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2192,7 +2192,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="44" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2214,7 +2214,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="45" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2236,7 +2236,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="46" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="G46" s="29"/>
     </row>
-    <row r="47" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2274,7 +2274,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="48" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2296,7 +2296,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="49" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2318,7 +2318,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="50" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2340,7 +2340,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="51" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2362,7 +2362,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="52" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2384,7 +2384,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="53" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2406,7 +2406,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="54" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2428,7 +2428,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="55" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2450,7 +2450,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="56" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B56" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2466,7 +2466,7 @@
       </c>
       <c r="G56" s="29"/>
     </row>
-    <row r="57" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2488,7 +2488,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="58" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B58" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2510,7 +2510,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="59" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B59" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2532,7 +2532,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="60" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B60" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2554,7 +2554,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="61" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2570,7 +2570,7 @@
       </c>
       <c r="G61" s="29"/>
     </row>
-    <row r="62" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2592,7 +2592,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="63" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B63" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2614,7 +2614,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="64" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B64" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2636,7 +2636,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="65" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B65" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2652,7 +2652,7 @@
       </c>
       <c r="G65" s="29"/>
     </row>
-    <row r="66" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2674,7 +2674,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="67" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2696,7 +2696,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="68" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B68" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2718,7 +2718,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="69" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B69" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2740,7 +2740,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="70" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B70" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="G70" s="29"/>
     </row>
-    <row r="71" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B71" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2778,7 +2778,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="72" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B72" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2800,7 +2800,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="73" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B73" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2822,7 +2822,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="74" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B74" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2844,7 +2844,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="75" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B75" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2866,7 +2866,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="76" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B76" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2882,7 +2882,7 @@
       </c>
       <c r="G76" s="29"/>
     </row>
-    <row r="77" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B77" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2904,7 +2904,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="78" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B78" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2926,7 +2926,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="79" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B79" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2948,7 +2948,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="80" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B80" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -2970,7 +2970,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="81" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B81" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="G81" s="29"/>
     </row>
-    <row r="82" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B82" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3008,7 +3008,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="83" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B83" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3030,7 +3030,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="84" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B84" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3052,7 +3052,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="85" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B85" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3074,7 +3074,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="86" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B86" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="G86" s="29"/>
     </row>
-    <row r="87" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B87" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3112,7 +3112,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="88" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B88" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3134,7 +3134,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="89" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B89" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3156,7 +3156,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="90" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B90" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3178,7 +3178,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="91" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B91" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3200,7 +3200,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="92" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B92" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3222,7 +3222,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="93" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B93" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3238,7 +3238,7 @@
       </c>
       <c r="G93" s="29"/>
     </row>
-    <row r="94" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B94" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3260,7 +3260,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="95" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B95" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3282,7 +3282,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="96" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B96" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3304,7 +3304,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="97" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B97" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3326,7 +3326,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="98" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B98" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="G98" s="29"/>
     </row>
-    <row r="99" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B99" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3364,7 +3364,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="100" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B100" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3386,7 +3386,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="101" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B101" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3408,7 +3408,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="102" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B102" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3430,7 +3430,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="103" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B103" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="G103" s="29"/>
     </row>
-    <row r="104" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B104" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3468,7 +3468,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="105" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B105" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3490,7 +3490,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="106" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B106" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3512,7 +3512,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="107" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B107" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3534,7 +3534,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="108" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B108" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3550,7 +3550,7 @@
       </c>
       <c r="G108" s="29"/>
     </row>
-    <row r="109" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B109" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3572,7 +3572,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="110" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B110" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3594,7 +3594,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="111" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B111" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3610,7 +3610,7 @@
       </c>
       <c r="G111" s="29"/>
     </row>
-    <row r="112" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B112" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3632,7 +3632,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="113" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B113" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3654,7 +3654,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="114" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B114" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3676,7 +3676,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="115" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B115" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3698,7 +3698,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="116" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B116" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3714,7 +3714,7 @@
       </c>
       <c r="G116" s="29"/>
     </row>
-    <row r="117" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B117" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3736,7 +3736,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="118" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B118" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3758,7 +3758,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="119" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B119" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="G119" s="29"/>
     </row>
-    <row r="120" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B120" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3796,7 +3796,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="121" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B121" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3818,7 +3818,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="122" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B122" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3840,7 +3840,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="123" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B123" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3862,7 +3862,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="124" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B124" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="G124" s="29"/>
     </row>
-    <row r="125" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B125" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3900,7 +3900,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="126" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B126" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3922,7 +3922,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="127" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B127" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3944,7 +3944,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="128" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B128" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3966,7 +3966,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="129" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B129" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -3988,7 +3988,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="130" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B130" s="11" t="str">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v/>
@@ -4004,7 +4004,7 @@
       </c>
       <c r="G130" s="29"/>
     </row>
-    <row r="131" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B131" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -4026,7 +4026,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="132" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B132" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>
@@ -4048,7 +4048,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="133" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B133" s="11">
         <f ca="1">Tasks[[#This Row],[Status Icon]]</f>
         <v>-1</v>

</xml_diff>